<commit_message>
SCRUM sprint 1 setup
</commit_message>
<xml_diff>
--- a/Docs/Scrum planning en rapport template.xlsx
+++ b/Docs/Scrum planning en rapport template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thecr\Documents\AP\2eJ-semester2\AI Project\AI-Project\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE03422A-7895-4DE6-8D1B-088C8AA5F088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8800475-A205-4BD5-B353-90BCF1D02C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{E07F6153-1B8C-43A7-97BD-457FD435295E}"/>
   </bookViews>
@@ -1284,8 +1284,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1295,6 +1293,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2449,30 +2449,30 @@
       <c r="B9" s="10"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
     </row>
     <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
     </row>
     <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
@@ -2490,12 +2490,12 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
+      <c r="F15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -2741,17 +2741,17 @@
       <c r="A35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
@@ -2883,18 +2883,24 @@
       <c r="A45" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="B35:J35"/>
     <mergeCell ref="B43:J43"/>
     <mergeCell ref="B44:J44"/>
     <mergeCell ref="B45:J45"/>
@@ -2904,12 +2910,6 @@
     <mergeCell ref="B40:J40"/>
     <mergeCell ref="B41:J41"/>
     <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="B35:J35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2990,30 +2990,30 @@
       <c r="B9" s="10"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
     </row>
     <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
     </row>
     <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
@@ -3031,12 +3031,12 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
+      <c r="F15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -3282,17 +3282,17 @@
       <c r="A35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
@@ -3424,18 +3424,24 @@
       <c r="A45" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="B35:J35"/>
     <mergeCell ref="B43:J43"/>
     <mergeCell ref="B44:J44"/>
     <mergeCell ref="B45:J45"/>
@@ -3445,12 +3451,6 @@
     <mergeCell ref="B40:J40"/>
     <mergeCell ref="B41:J41"/>
     <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="B35:J35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -5134,32 +5134,32 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
     </row>
     <row r="12" spans="1:13" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
     </row>
     <row r="14" spans="1:13" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
@@ -5177,12 +5177,12 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
+      <c r="F15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
       <c r="L15" s="2" t="s">
         <v>7</v>
       </c>
@@ -5241,8 +5241,8 @@
       <c r="D17" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E17" t="s">
-        <v>16</v>
+      <c r="E17" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="F17" s="3">
         <v>9.5</v>
@@ -5277,7 +5277,7 @@
       <c r="D18" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F18" s="3"/>
@@ -5301,7 +5301,7 @@
       <c r="D19" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="3" t="s">
         <v>17</v>
       </c>
       <c r="F19" s="3">
@@ -5329,8 +5329,8 @@
       <c r="D20" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E20" t="s">
-        <v>15</v>
+      <c r="E20" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3">
@@ -5353,8 +5353,8 @@
       <c r="D21" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="E21" t="s">
-        <v>16</v>
+      <c r="E21" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="F21" s="3">
         <v>2</v>
@@ -5377,8 +5377,8 @@
       <c r="D22" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E22" t="s">
-        <v>15</v>
+      <c r="E22" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -5401,10 +5401,12 @@
       <c r="D23" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E23" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="3"/>
+      <c r="E23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="3">
+        <v>1</v>
+      </c>
       <c r="G23" s="3"/>
       <c r="H23" s="3">
         <v>6</v>
@@ -5425,8 +5427,8 @@
       <c r="D24" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E24" t="s">
-        <v>15</v>
+      <c r="E24" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3">
@@ -5450,10 +5452,10 @@
         <v>165</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F25" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
@@ -5564,17 +5566,17 @@
       <c r="A35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
@@ -5706,15 +5708,1097 @@
       <c r="A45" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B43:J43"/>
+    <mergeCell ref="B44:J44"/>
+    <mergeCell ref="B45:J45"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B39:J39"/>
+    <mergeCell ref="B40:J40"/>
+    <mergeCell ref="B41:J41"/>
+    <mergeCell ref="B42:J42"/>
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="B35:J35"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88C0E642-EED7-4937-B528-376AB48F1EE7}">
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="5" width="17.77734375" customWidth="1"/>
+    <col min="6" max="9" width="10.77734375" customWidth="1"/>
+    <col min="10" max="10" width="35.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+    </row>
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="10"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="10"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="10"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="10"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="10"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
+    </row>
+    <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
+    </row>
+    <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="2"/>
+      <c r="F15" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="5">
+        <f>SUM(F17:F30)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="5">
+        <f t="shared" ref="G31:I31" si="0">SUM(G17:G30)</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I31" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J31" s="5"/>
+    </row>
+    <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B36" s="38"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
+      <c r="J36" s="39"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="38"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="38"/>
+      <c r="J37" s="39"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B38" s="38"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+      <c r="J38" s="39"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A39" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" s="38"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
+      <c r="J39" s="39"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B40" s="38"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="38"/>
+      <c r="J40" s="39"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A41" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B41" s="38"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="38"/>
+      <c r="J41" s="39"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A42" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B42" s="38"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="38"/>
+      <c r="J42" s="39"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A43" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B43" s="38"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="38"/>
+      <c r="J43" s="39"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A44" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="38"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="38"/>
+      <c r="J44" s="39"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A45" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B43:J43"/>
+    <mergeCell ref="B44:J44"/>
+    <mergeCell ref="B45:J45"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B39:J39"/>
+    <mergeCell ref="B40:J40"/>
+    <mergeCell ref="B41:J41"/>
+    <mergeCell ref="B42:J42"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE36C8E1-C9DA-45BD-B73B-7521063AD367}">
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
+    <col min="3" max="3" width="12.44140625" customWidth="1"/>
+    <col min="4" max="5" width="17.77734375" customWidth="1"/>
+    <col min="6" max="9" width="10.77734375" customWidth="1"/>
+    <col min="10" max="10" width="35.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+    </row>
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="10"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="10"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="10"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="10"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="10"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
+    </row>
+    <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
+    </row>
+    <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="2"/>
+      <c r="F15" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="5">
+        <f>SUM(F17:F30)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="5">
+        <f t="shared" ref="G31:I31" si="0">SUM(G17:G30)</f>
+        <v>0</v>
+      </c>
+      <c r="H31" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I31" s="5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J31" s="5"/>
+    </row>
+    <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B36" s="38"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
+      <c r="J36" s="39"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="38"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="38"/>
+      <c r="J37" s="39"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B38" s="38"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+      <c r="J38" s="39"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A39" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" s="38"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
+      <c r="J39" s="39"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B40" s="38"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="38"/>
+      <c r="J40" s="39"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A41" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B41" s="38"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="38"/>
+      <c r="J41" s="39"/>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A42" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B42" s="38"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="38"/>
+      <c r="J42" s="39"/>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A43" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B43" s="38"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="38"/>
+      <c r="J43" s="39"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A44" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="38"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="38"/>
+      <c r="J44" s="39"/>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A45" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -5741,1088 +6825,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88C0E642-EED7-4937-B528-376AB48F1EE7}">
-  <dimension ref="A1:J45"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.77734375" customWidth="1"/>
-    <col min="2" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="5" width="17.77734375" customWidth="1"/>
-    <col min="6" max="9" width="10.77734375" customWidth="1"/>
-    <col min="10" max="10" width="35.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-    </row>
-    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="10"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="10"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="10"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="10"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="10"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
-    </row>
-    <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-    </row>
-    <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="5">
-        <f>SUM(F17:F30)</f>
-        <v>0</v>
-      </c>
-      <c r="G31" s="5">
-        <f t="shared" ref="G31:I31" si="0">SUM(G17:G30)</f>
-        <v>0</v>
-      </c>
-      <c r="H31" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I31" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J31" s="5"/>
-    </row>
-    <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="45" t="s">
-        <v>54</v>
-      </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="B36" s="38"/>
-      <c r="C36" s="38"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
-      <c r="H36" s="38"/>
-      <c r="I36" s="38"/>
-      <c r="J36" s="39"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B37" s="38"/>
-      <c r="C37" s="38"/>
-      <c r="D37" s="38"/>
-      <c r="E37" s="38"/>
-      <c r="F37" s="38"/>
-      <c r="G37" s="38"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="38"/>
-      <c r="J37" s="39"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B38" s="38"/>
-      <c r="C38" s="38"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="38"/>
-      <c r="F38" s="38"/>
-      <c r="G38" s="38"/>
-      <c r="H38" s="38"/>
-      <c r="I38" s="38"/>
-      <c r="J38" s="39"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B39" s="38"/>
-      <c r="C39" s="38"/>
-      <c r="D39" s="38"/>
-      <c r="E39" s="38"/>
-      <c r="F39" s="38"/>
-      <c r="G39" s="38"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="38"/>
-      <c r="J39" s="39"/>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B40" s="38"/>
-      <c r="C40" s="38"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="38"/>
-      <c r="F40" s="38"/>
-      <c r="G40" s="38"/>
-      <c r="H40" s="38"/>
-      <c r="I40" s="38"/>
-      <c r="J40" s="39"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B41" s="38"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="38"/>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
-      <c r="I41" s="38"/>
-      <c r="J41" s="39"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="B42" s="38"/>
-      <c r="C42" s="38"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
-      <c r="H42" s="38"/>
-      <c r="I42" s="38"/>
-      <c r="J42" s="39"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B43" s="38"/>
-      <c r="C43" s="38"/>
-      <c r="D43" s="38"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="38"/>
-      <c r="G43" s="38"/>
-      <c r="H43" s="38"/>
-      <c r="I43" s="38"/>
-      <c r="J43" s="39"/>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="B44" s="38"/>
-      <c r="C44" s="38"/>
-      <c r="D44" s="38"/>
-      <c r="E44" s="38"/>
-      <c r="F44" s="38"/>
-      <c r="G44" s="38"/>
-      <c r="H44" s="38"/>
-      <c r="I44" s="38"/>
-      <c r="J44" s="39"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A45" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
-    </row>
-  </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="B43:J43"/>
-    <mergeCell ref="B44:J44"/>
-    <mergeCell ref="B45:J45"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="B38:J38"/>
-    <mergeCell ref="B39:J39"/>
-    <mergeCell ref="B40:J40"/>
-    <mergeCell ref="B41:J41"/>
-    <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="B35:J35"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE36C8E1-C9DA-45BD-B73B-7521063AD367}">
-  <dimension ref="A1:J45"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="16.77734375" customWidth="1"/>
-    <col min="2" max="2" width="38" customWidth="1"/>
-    <col min="3" max="3" width="12.44140625" customWidth="1"/>
-    <col min="4" max="5" width="17.77734375" customWidth="1"/>
-    <col min="6" max="9" width="10.77734375" customWidth="1"/>
-    <col min="10" max="10" width="35.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-    </row>
-    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="10"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="10"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="10"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="10"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="10"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
-    </row>
-    <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-    </row>
-    <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A14" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="I16" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="5">
-        <f>SUM(F17:F30)</f>
-        <v>0</v>
-      </c>
-      <c r="G31" s="5">
-        <f t="shared" ref="G31:I31" si="0">SUM(G17:G30)</f>
-        <v>0</v>
-      </c>
-      <c r="H31" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I31" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J31" s="5"/>
-    </row>
-    <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="A33" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="45" t="s">
-        <v>54</v>
-      </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="B36" s="38"/>
-      <c r="C36" s="38"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="38"/>
-      <c r="F36" s="38"/>
-      <c r="G36" s="38"/>
-      <c r="H36" s="38"/>
-      <c r="I36" s="38"/>
-      <c r="J36" s="39"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B37" s="38"/>
-      <c r="C37" s="38"/>
-      <c r="D37" s="38"/>
-      <c r="E37" s="38"/>
-      <c r="F37" s="38"/>
-      <c r="G37" s="38"/>
-      <c r="H37" s="38"/>
-      <c r="I37" s="38"/>
-      <c r="J37" s="39"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B38" s="38"/>
-      <c r="C38" s="38"/>
-      <c r="D38" s="38"/>
-      <c r="E38" s="38"/>
-      <c r="F38" s="38"/>
-      <c r="G38" s="38"/>
-      <c r="H38" s="38"/>
-      <c r="I38" s="38"/>
-      <c r="J38" s="39"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B39" s="38"/>
-      <c r="C39" s="38"/>
-      <c r="D39" s="38"/>
-      <c r="E39" s="38"/>
-      <c r="F39" s="38"/>
-      <c r="G39" s="38"/>
-      <c r="H39" s="38"/>
-      <c r="I39" s="38"/>
-      <c r="J39" s="39"/>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B40" s="38"/>
-      <c r="C40" s="38"/>
-      <c r="D40" s="38"/>
-      <c r="E40" s="38"/>
-      <c r="F40" s="38"/>
-      <c r="G40" s="38"/>
-      <c r="H40" s="38"/>
-      <c r="I40" s="38"/>
-      <c r="J40" s="39"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B41" s="38"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="38"/>
-      <c r="F41" s="38"/>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
-      <c r="I41" s="38"/>
-      <c r="J41" s="39"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="B42" s="38"/>
-      <c r="C42" s="38"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="38"/>
-      <c r="F42" s="38"/>
-      <c r="G42" s="38"/>
-      <c r="H42" s="38"/>
-      <c r="I42" s="38"/>
-      <c r="J42" s="39"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B43" s="38"/>
-      <c r="C43" s="38"/>
-      <c r="D43" s="38"/>
-      <c r="E43" s="38"/>
-      <c r="F43" s="38"/>
-      <c r="G43" s="38"/>
-      <c r="H43" s="38"/>
-      <c r="I43" s="38"/>
-      <c r="J43" s="39"/>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="B44" s="38"/>
-      <c r="C44" s="38"/>
-      <c r="D44" s="38"/>
-      <c r="E44" s="38"/>
-      <c r="F44" s="38"/>
-      <c r="G44" s="38"/>
-      <c r="H44" s="38"/>
-      <c r="I44" s="38"/>
-      <c r="J44" s="39"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A45" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
-    </row>
-  </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="B43:J43"/>
-    <mergeCell ref="B44:J44"/>
-    <mergeCell ref="B45:J45"/>
-    <mergeCell ref="B37:J37"/>
-    <mergeCell ref="B38:J38"/>
-    <mergeCell ref="B39:J39"/>
-    <mergeCell ref="B40:J40"/>
-    <mergeCell ref="B41:J41"/>
-    <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="B35:J35"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7DDB97A-7F06-4418-A020-7176AC18CA0E}">
   <dimension ref="A1:J45"/>
@@ -6895,30 +6897,30 @@
       <c r="B9" s="10"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
     </row>
     <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
     </row>
     <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
@@ -6936,12 +6938,12 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
+      <c r="F15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -7187,17 +7189,17 @@
       <c r="A35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
@@ -7329,18 +7331,24 @@
       <c r="A45" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="B35:J35"/>
     <mergeCell ref="B43:J43"/>
     <mergeCell ref="B44:J44"/>
     <mergeCell ref="B45:J45"/>
@@ -7350,12 +7358,6 @@
     <mergeCell ref="B40:J40"/>
     <mergeCell ref="B41:J41"/>
     <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="B35:J35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -7436,30 +7438,30 @@
       <c r="B9" s="10"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
     </row>
     <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
     </row>
     <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
@@ -7477,12 +7479,12 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
+      <c r="F15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -7728,17 +7730,17 @@
       <c r="A35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
@@ -7870,18 +7872,24 @@
       <c r="A45" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="B35:J35"/>
     <mergeCell ref="B43:J43"/>
     <mergeCell ref="B44:J44"/>
     <mergeCell ref="B45:J45"/>
@@ -7891,12 +7899,6 @@
     <mergeCell ref="B40:J40"/>
     <mergeCell ref="B41:J41"/>
     <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="B35:J35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -7977,30 +7979,30 @@
       <c r="B9" s="10"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="42"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="40"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="40"/>
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
     </row>
     <row r="12" spans="1:10" ht="43.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="43"/>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
+      <c r="A12" s="41"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="41"/>
+      <c r="H12" s="41"/>
+      <c r="I12" s="41"/>
+      <c r="J12" s="41"/>
     </row>
     <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
@@ -8018,12 +8020,12 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="F15" s="44" t="s">
+      <c r="F15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
-      <c r="I15" s="44"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="42"/>
+      <c r="I15" s="42"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -8269,17 +8271,17 @@
       <c r="A35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="45" t="s">
+      <c r="B35" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45"/>
-      <c r="H35" s="45"/>
-      <c r="I35" s="45"/>
-      <c r="J35" s="46"/>
+      <c r="C35" s="43"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="43"/>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+      <c r="H35" s="43"/>
+      <c r="I35" s="43"/>
+      <c r="J35" s="44"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
@@ -8411,18 +8413,24 @@
       <c r="A45" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40"/>
-      <c r="F45" s="40"/>
-      <c r="G45" s="40"/>
-      <c r="H45" s="40"/>
-      <c r="I45" s="40"/>
-      <c r="J45" s="41"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
+      <c r="E45" s="45"/>
+      <c r="F45" s="45"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="45"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="46"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A11:J11"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="B35:J35"/>
     <mergeCell ref="B43:J43"/>
     <mergeCell ref="B44:J44"/>
     <mergeCell ref="B45:J45"/>
@@ -8432,12 +8440,6 @@
     <mergeCell ref="B40:J40"/>
     <mergeCell ref="B41:J41"/>
     <mergeCell ref="B42:J42"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="B35:J35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -8447,6 +8449,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009EB83581AE75E3448E2425BE2C4A9358" ma:contentTypeVersion="2" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="3613ffd620ebef032c0b03220f523539">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87f001ec-f7b3-49be-8676-481a173a404e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="972cec87c5ab16132ba820573bf22a25" ns2:_="">
     <xsd:import namespace="87f001ec-f7b3-49be-8676-481a173a404e"/>
@@ -8578,12 +8586,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -8594,6 +8596,22 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{959E2576-8ACA-4472-AE2B-4AF07B9AFF6B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="87f001ec-f7b3-49be-8676-481a173a404e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5025CB3-4618-43BF-8CBB-8A6ABF966F86}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8611,22 +8629,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{959E2576-8ACA-4472-AE2B-4AF07B9AFF6B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="87f001ec-f7b3-49be-8676-481a173a404e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{05AA98B7-DD2A-4000-A348-80CCBB56207C}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
added init.sql schema and updated compose for account creation (GH-08)
</commit_message>
<xml_diff>
--- a/Docs/Scrum planning en rapport template.xlsx
+++ b/Docs/Scrum planning en rapport template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thecr\Documents\AP\2eJ-semester2\AI Project\AI-Project\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8800475-A205-4BD5-B353-90BCF1D02C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518AF41C-4D30-4AA6-8D60-665D5F70FF5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{E07F6153-1B8C-43A7-97BD-457FD435295E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{E07F6153-1B8C-43A7-97BD-457FD435295E}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="3" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="227">
   <si>
     <t>Dashboard</t>
   </si>
@@ -526,9 +526,6 @@
     <t>Model (her)training</t>
   </si>
   <si>
-    <t>Hertraining model</t>
-  </si>
-  <si>
     <t>Als beheerder wil ik een versiebeheer van mijn model zodat ik een ander versie kan gebruiken.</t>
   </si>
   <si>
@@ -763,9 +760,6 @@
     <t>GH-33</t>
   </si>
   <si>
-    <t>GH-4, GH-5,  GH-24 &amp; GH-34</t>
-  </si>
-  <si>
     <t>GH-29 &amp; GH-30</t>
   </si>
   <si>
@@ -833,6 +827,12 @@
   </si>
   <si>
     <t>Optioneel? We hebben hiervoor geen userstories.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GH-4, GH-5,  GH-24 </t>
+  </si>
+  <si>
+    <t>(Her)training model</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1195,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1295,6 +1295,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1742,8 +1745,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C31D63E-5C3E-42E3-BE92-09D26924F40D}" name="Table1" displayName="Table1" ref="A3:J36" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
-  <autoFilter ref="A3:J36" xr:uid="{0C31D63E-5C3E-42E3-BE92-09D26924F40D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0C31D63E-5C3E-42E3-BE92-09D26924F40D}" name="Table1" displayName="Table1" ref="A3:J37" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
+  <autoFilter ref="A3:J37" xr:uid="{0C31D63E-5C3E-42E3-BE92-09D26924F40D}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:J36">
     <sortCondition ref="A3:A36"/>
   </sortState>
@@ -2223,7 +2226,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D3" s="33"/>
     </row>
@@ -3659,7 +3662,7 @@
         <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D12" s="17" t="s">
         <v>83</v>
@@ -3673,7 +3676,7 @@
         <v>78</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D13" s="17" t="s">
         <v>83</v>
@@ -3687,7 +3690,7 @@
         <v>79</v>
       </c>
       <c r="C14" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D14" s="17" t="s">
         <v>83</v>
@@ -3701,13 +3704,13 @@
         <v>80</v>
       </c>
       <c r="C15" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>88</v>
       </c>
       <c r="E15" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -3718,7 +3721,7 @@
         <v>81</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>83</v>
@@ -3732,7 +3735,7 @@
         <v>82</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>83</v>
@@ -3746,7 +3749,7 @@
         <v>91</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D18" s="17" t="s">
         <v>83</v>
@@ -3761,7 +3764,7 @@
         <v>95</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D19" s="18" t="s">
         <v>83</v>
@@ -3769,13 +3772,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>146</v>
+      </c>
+      <c r="B20" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="B20" s="27" t="s">
-        <v>148</v>
-      </c>
       <c r="C20" s="17" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D20" s="17" t="s">
         <v>83</v>
@@ -3787,10 +3790,10 @@
         <v>87</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D21" s="17" t="s">
         <v>96</v>
@@ -3799,13 +3802,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>85</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D22" s="18" t="s">
         <v>83</v>
@@ -3817,10 +3820,10 @@
         <v>94</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C23" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D23" t="s">
         <v>88</v>
@@ -3834,7 +3837,7 @@
         <v>92</v>
       </c>
       <c r="C24" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D24" t="s">
         <v>88</v>
@@ -3999,7 +4002,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8A4E451-46AC-4478-9EE0-DA5C244416C9}">
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" customWidth="1"/>
@@ -4077,13 +4080,13 @@
         <v>91</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G4" s="3">
         <v>5</v>
@@ -4099,7 +4102,7 @@
     </row>
     <row r="5" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>108</v>
@@ -4108,13 +4111,13 @@
         <v>77</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G5" s="3">
         <v>5</v>
@@ -4130,7 +4133,7 @@
     </row>
     <row r="6" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>109</v>
@@ -4159,10 +4162,10 @@
     </row>
     <row r="7" spans="1:12" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>78</v>
@@ -4191,10 +4194,10 @@
     </row>
     <row r="8" spans="1:12" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C8" s="19" t="s">
         <v>78</v>
@@ -4223,22 +4226,22 @@
     </row>
     <row r="9" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C9" s="23" t="s">
         <v>78</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="G9" s="3">
         <v>13</v>
@@ -4254,7 +4257,7 @@
     </row>
     <row r="10" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>110</v>
@@ -4263,7 +4266,7 @@
         <v>79</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>34</v>
@@ -4286,7 +4289,7 @@
     </row>
     <row r="11" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>111</v>
@@ -4301,7 +4304,7 @@
         <v>33</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G11" s="3">
         <v>2</v>
@@ -4314,7 +4317,7 @@
     </row>
     <row r="12" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>113</v>
@@ -4343,10 +4346,10 @@
     </row>
     <row r="13" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>79</v>
@@ -4372,7 +4375,7 @@
     </row>
     <row r="14" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>120</v>
@@ -4401,7 +4404,7 @@
     </row>
     <row r="15" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>121</v>
@@ -4430,7 +4433,7 @@
     </row>
     <row r="16" spans="1:12" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>122</v>
@@ -4459,16 +4462,16 @@
     </row>
     <row r="17" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>124</v>
+        <v>226</v>
       </c>
       <c r="C17" s="29" t="s">
         <v>82</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>32</v>
@@ -4488,16 +4491,16 @@
     </row>
     <row r="18" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C18" s="24" t="s">
         <v>82</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>33</v>
@@ -4517,7 +4520,7 @@
     </row>
     <row r="19" spans="1:10" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>99</v>
@@ -4546,7 +4549,7 @@
     </row>
     <row r="20" spans="1:10" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>101</v>
@@ -4575,7 +4578,7 @@
     </row>
     <row r="21" spans="1:10" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>105</v>
@@ -4584,13 +4587,13 @@
         <v>91</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G21" s="3">
         <v>8</v>
@@ -4603,22 +4606,22 @@
     </row>
     <row r="22" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C22" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G22" s="3">
         <v>8</v>
@@ -4631,22 +4634,22 @@
     </row>
     <row r="23" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G23" s="3">
         <v>0.5</v>
@@ -4659,22 +4662,22 @@
     </row>
     <row r="24" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C24" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G24" s="3">
         <v>1</v>
@@ -4687,22 +4690,22 @@
     </row>
     <row r="25" spans="1:10" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C25" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G25" s="3">
         <v>1</v>
@@ -4715,22 +4718,22 @@
     </row>
     <row r="26" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C26" s="24" t="s">
         <v>95</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>33</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G26" s="3">
         <v>3</v>
@@ -4743,22 +4746,22 @@
     </row>
     <row r="27" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>157</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G27" s="3">
         <v>5</v>
@@ -4771,22 +4774,22 @@
     </row>
     <row r="28" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G28" s="3">
         <v>8</v>
@@ -4799,22 +4802,22 @@
     </row>
     <row r="29" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G29" s="3">
         <v>5</v>
@@ -4827,22 +4830,22 @@
     </row>
     <row r="30" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C30" s="22" t="s">
         <v>85</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G30" s="3">
         <v>2</v>
@@ -4855,22 +4858,22 @@
     </row>
     <row r="31" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C31" s="22" t="s">
         <v>85</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>33</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G31" s="3">
         <v>13</v>
@@ -4883,22 +4886,22 @@
     </row>
     <row r="32" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C32" s="22" t="s">
         <v>85</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G32" s="3">
         <v>5</v>
@@ -4911,22 +4914,22 @@
     </row>
     <row r="33" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C33" s="26" t="s">
         <v>85</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>33</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G33" s="3">
         <v>1</v>
@@ -4939,22 +4942,22 @@
     </row>
     <row r="34" spans="1:10" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B34" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C34" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="C34" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>150</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>33</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G34" s="3">
         <v>5</v>
@@ -4967,22 +4970,22 @@
     </row>
     <row r="35" spans="1:10" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C35" s="24" t="s">
         <v>92</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G35" s="3">
         <v>8</v>
@@ -4995,22 +4998,22 @@
     </row>
     <row r="36" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C36" s="24" t="s">
         <v>92</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>34</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G36" s="3">
         <v>8</v>
@@ -5020,6 +5023,21 @@
         <v>15</v>
       </c>
       <c r="J36" s="3"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="47" t="str">
+        <f>A36</f>
+        <v>GH-33</v>
+      </c>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5027,10 +5045,10 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4:I36" xr:uid="{BB889DD1-88CD-4BDB-98A5-3CC9C5D63332}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4:I37" xr:uid="{BB889DD1-88CD-4BDB-98A5-3CC9C5D63332}">
       <formula1>$L$3:$L$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E36" xr:uid="{D4954F6E-5C80-4868-8B20-BF00C35F9218}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E37" xr:uid="{D4954F6E-5C80-4868-8B20-BF00C35F9218}">
       <formula1>$L$8:$L$10</formula1>
     </dataValidation>
   </dataValidations>
@@ -5127,6 +5145,7 @@
         <v>42</v>
       </c>
       <c r="B9" s="10">
+        <f>SUM(C17:C25)</f>
         <v>32</v>
       </c>
       <c r="L9" t="s">
@@ -5230,16 +5249,16 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C17" s="3">
         <v>8</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>17</v>
@@ -5255,7 +5274,7 @@
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>9</v>
@@ -5266,16 +5285,16 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C18" s="3">
         <v>0.5</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>17</v>
@@ -5290,16 +5309,16 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C19" s="3">
         <v>1</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>17</v>
@@ -5318,16 +5337,16 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C20" s="3">
         <v>1</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>17</v>
@@ -5342,16 +5361,16 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C21" s="3">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>17</v>
@@ -5366,7 +5385,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>101</v>
@@ -5375,7 +5394,7 @@
         <v>0.5</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>17</v>
@@ -5390,7 +5409,7 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>105</v>
@@ -5399,7 +5418,7 @@
         <v>8</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>17</v>
@@ -5416,7 +5435,7 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>99</v>
@@ -5425,7 +5444,7 @@
         <v>5</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>17</v>
@@ -5449,7 +5468,7 @@
         <v>5</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>17</v>
@@ -5788,19 +5807,25 @@
       <c r="A5" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="10"/>
+      <c r="B5" s="21">
+        <v>46076</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="21">
+        <v>46090</v>
+      </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="10">
+        <v>2</v>
+      </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
@@ -5896,8 +5921,12 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+      <c r="A17" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>159</v>
+      </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -5908,7 +5937,9 @@
       <c r="J17" s="3"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>174</v>
+      </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -5920,8 +5951,12 @@
       <c r="J18" s="3"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+      <c r="A19" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>155</v>
+      </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
@@ -5932,8 +5967,12 @@
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+      <c r="A20" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>

</xml_diff>